<commit_message>
TC-AuthN-01 test case completed
</commit_message>
<xml_diff>
--- a/docs/testing/rtm.xlsx
+++ b/docs/testing/rtm.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="122">
   <si>
     <t xml:space="preserve">Requirement ID</t>
   </si>
@@ -70,16 +70,13 @@
     <t xml:space="preserve">Unit (Front)</t>
   </si>
   <si>
-    <t xml:space="preserve">In Execution</t>
+    <t xml:space="preserve">Passed</t>
   </si>
   <si>
     <t xml:space="preserve">TC-AuthN-02</t>
   </si>
   <si>
     <t xml:space="preserve">Unit (Back)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passed</t>
   </si>
   <si>
     <t xml:space="preserve">TC-AuthN-03</t>
@@ -615,34 +612,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -784,7 +781,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I67"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="41.3"/>
@@ -793,7 +790,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="17.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="17.88"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -865,7 +862,7 @@
         <v>18</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I3" s="5"/>
     </row>
@@ -876,13 +873,13 @@
       <c r="D4" s="6"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I4" s="5"/>
     </row>
@@ -893,13 +890,13 @@
       <c r="D5" s="6"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I5" s="5"/>
     </row>
@@ -910,13 +907,13 @@
       <c r="D6" s="6"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>25</v>
-      </c>
       <c r="H6" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I6" s="5"/>
     </row>
@@ -927,22 +924,22 @@
       <c r="D7" s="6"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>11</v>
@@ -954,13 +951,13 @@
         <v>13</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I8" s="5"/>
     </row>
@@ -971,13 +968,13 @@
       <c r="D9" s="6"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I9" s="5"/>
     </row>
@@ -988,13 +985,13 @@
       <c r="D10" s="6"/>
       <c r="E10" s="5"/>
       <c r="F10" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I10" s="5"/>
     </row>
@@ -1005,13 +1002,13 @@
       <c r="D11" s="6"/>
       <c r="E11" s="5"/>
       <c r="F11" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I11" s="5"/>
     </row>
@@ -1022,13 +1019,13 @@
       <c r="D12" s="6"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I12" s="5"/>
     </row>
@@ -1039,22 +1036,22 @@
       <c r="D13" s="6"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>11</v>
@@ -1066,13 +1063,13 @@
         <v>13</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I14" s="5"/>
     </row>
@@ -1083,13 +1080,13 @@
       <c r="D15" s="6"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I15" s="5"/>
     </row>
@@ -1100,13 +1097,13 @@
       <c r="D16" s="6"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I16" s="5"/>
     </row>
@@ -1117,13 +1114,13 @@
       <c r="D17" s="6"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I17" s="5"/>
     </row>
@@ -1134,13 +1131,13 @@
       <c r="D18" s="6"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I18" s="5"/>
     </row>
@@ -1151,22 +1148,22 @@
       <c r="D19" s="6"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>11</v>
@@ -1178,13 +1175,13 @@
         <v>13</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I20" s="5"/>
     </row>
@@ -1195,13 +1192,13 @@
       <c r="D21" s="6"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I21" s="5"/>
     </row>
@@ -1212,13 +1209,13 @@
       <c r="D22" s="6"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I22" s="5"/>
     </row>
@@ -1229,13 +1226,13 @@
       <c r="D23" s="6"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I23" s="5"/>
     </row>
@@ -1246,22 +1243,22 @@
       <c r="D24" s="6"/>
       <c r="E24" s="5"/>
       <c r="F24" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>11</v>
@@ -1273,13 +1270,13 @@
         <v>13</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I25" s="5"/>
     </row>
@@ -1290,13 +1287,13 @@
       <c r="D26" s="6"/>
       <c r="E26" s="5"/>
       <c r="F26" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I26" s="5"/>
     </row>
@@ -1307,13 +1304,13 @@
       <c r="D27" s="6"/>
       <c r="E27" s="5"/>
       <c r="F27" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I27" s="5"/>
     </row>
@@ -1324,22 +1321,22 @@
       <c r="D28" s="6"/>
       <c r="E28" s="5"/>
       <c r="F28" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>57</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>11</v>
@@ -1351,13 +1348,13 @@
         <v>13</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I29" s="5"/>
     </row>
@@ -1368,13 +1365,13 @@
       <c r="D30" s="6"/>
       <c r="E30" s="5"/>
       <c r="F30" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I30" s="5"/>
     </row>
@@ -1385,13 +1382,13 @@
       <c r="D31" s="6"/>
       <c r="E31" s="5"/>
       <c r="F31" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I31" s="5"/>
     </row>
@@ -1402,13 +1399,13 @@
       <c r="D32" s="6"/>
       <c r="E32" s="5"/>
       <c r="F32" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I32" s="5"/>
     </row>
@@ -1419,13 +1416,13 @@
       <c r="D33" s="6"/>
       <c r="E33" s="5"/>
       <c r="F33" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I33" s="5"/>
     </row>
@@ -1436,22 +1433,22 @@
       <c r="D34" s="6"/>
       <c r="E34" s="5"/>
       <c r="F34" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>11</v>
@@ -1463,13 +1460,13 @@
         <v>13</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I35" s="5"/>
     </row>
@@ -1480,13 +1477,13 @@
       <c r="D36" s="6"/>
       <c r="E36" s="5"/>
       <c r="F36" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I36" s="5"/>
     </row>
@@ -1497,13 +1494,13 @@
       <c r="D37" s="6"/>
       <c r="E37" s="5"/>
       <c r="F37" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I37" s="5"/>
     </row>
@@ -1514,13 +1511,13 @@
       <c r="D38" s="6"/>
       <c r="E38" s="5"/>
       <c r="F38" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I38" s="5"/>
     </row>
@@ -1531,40 +1528,40 @@
       <c r="D39" s="6"/>
       <c r="E39" s="5"/>
       <c r="F39" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>72</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I40" s="5"/>
     </row>
@@ -1575,13 +1572,13 @@
       <c r="D41" s="6"/>
       <c r="E41" s="5"/>
       <c r="F41" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I41" s="5"/>
     </row>
@@ -1592,13 +1589,13 @@
       <c r="D42" s="6"/>
       <c r="E42" s="5"/>
       <c r="F42" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I42" s="5"/>
     </row>
@@ -1609,13 +1606,13 @@
       <c r="D43" s="6"/>
       <c r="E43" s="5"/>
       <c r="F43" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I43" s="5"/>
     </row>
@@ -1626,40 +1623,40 @@
       <c r="D44" s="6"/>
       <c r="E44" s="5"/>
       <c r="F44" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>80</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E45" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I45" s="5"/>
     </row>
@@ -1670,13 +1667,13 @@
       <c r="D46" s="6"/>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I46" s="5"/>
     </row>
@@ -1687,40 +1684,40 @@
       <c r="D47" s="6"/>
       <c r="E47" s="5"/>
       <c r="F47" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I48" s="5"/>
     </row>
@@ -1731,13 +1728,13 @@
       <c r="D49" s="6"/>
       <c r="E49" s="5"/>
       <c r="F49" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I49" s="5"/>
     </row>
@@ -1748,13 +1745,13 @@
       <c r="D50" s="6"/>
       <c r="E50" s="5"/>
       <c r="F50" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I50" s="5"/>
     </row>
@@ -1765,13 +1762,13 @@
       <c r="D51" s="6"/>
       <c r="E51" s="5"/>
       <c r="F51" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I51" s="5"/>
     </row>
@@ -1782,40 +1779,40 @@
       <c r="D52" s="6"/>
       <c r="E52" s="5"/>
       <c r="F52" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B53" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>92</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E53" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I53" s="5"/>
     </row>
@@ -1826,13 +1823,13 @@
       <c r="D54" s="6"/>
       <c r="E54" s="5"/>
       <c r="F54" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I54" s="5"/>
     </row>
@@ -1843,40 +1840,40 @@
       <c r="D55" s="6"/>
       <c r="E55" s="5"/>
       <c r="F55" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G55" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B56" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>97</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I56" s="5"/>
     </row>
@@ -1887,243 +1884,243 @@
       <c r="D57" s="6"/>
       <c r="E57" s="5"/>
       <c r="F57" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B58" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D58" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E58" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
       <c r="H58" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D59" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E59" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
       <c r="H59" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D60" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E60" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
       <c r="H60" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D61" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E61" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="F61" s="5"/>
       <c r="G61" s="5"/>
       <c r="H61" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D62" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E62" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="E62" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
       <c r="H62" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="C63" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F63" s="5"/>
       <c r="G63" s="5"/>
       <c r="H63" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B64" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>116</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B65" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="C65" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F65" s="5"/>
       <c r="G65" s="5"/>
       <c r="H65" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B66" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="B66" s="5" t="s">
-        <v>120</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F66" s="5"/>
       <c r="G66" s="5"/>
       <c r="H66" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B67" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="B67" s="8" t="s">
-        <v>122</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F67" s="8"/>
       <c r="G67" s="8"/>
       <c r="H67" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I67" s="8"/>
     </row>

</xml_diff>